<commit_message>
Fix segment cancellation calculation and dashboard findings
</commit_message>
<xml_diff>
--- a/excel/Subscription_Churn_Retention_Analytics.xlsx
+++ b/excel/Subscription_Churn_Retention_Analytics.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R7aa717e3bbb24475"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Data" sheetId="2" r:id="R535e327da7e74d3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Trends" sheetId="3" r:id="Rfef218bea5364b80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan Performance" sheetId="4" r:id="R3afc74226faa4760"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cancellation Reasons" sheetId="5" r:id="R96f4b55a00a34222"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segment Analysis" sheetId="6" r:id="R988dddf33bb244cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohort Retention" sheetId="7" r:id="R4bc5381a8674434b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Definitions" sheetId="8" r:id="Rc2a2bec578cf4b72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5e0718605e894155"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Data" sheetId="2" r:id="Rd0c02664647a49dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Trends" sheetId="3" r:id="Re1cd77af1fb04a96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan Performance" sheetId="4" r:id="Rd599e29d01a74019"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cancellation Reasons" sheetId="5" r:id="R34489a746df04701"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segment Analysis" sheetId="6" r:id="R17a6d1e935574131"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohort Retention" sheetId="7" r:id="Ra0bd44f1a6c3404b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Definitions" sheetId="8" r:id="R97c64b92a70d43cb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -233,7 +233,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="200">
+  <x:cellXfs count="201">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -650,6 +650,7 @@
     <x:xf numFmtId="203" fontId="19" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -666,6 +667,7 @@
       <c:layout/>
       <c:lineChart>
         <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
@@ -983,7 +985,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R74b2554692e5445b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcd1f790722764238"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1013,7 +1015,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R68271bcbbad948ba"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R83de476f894f4b4e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1845,7 +1847,7 @@
       <x:c r="A32" s="178" t="str">
         <x:v>• Highest current cancelled share: Basic (35.3%).
 • Most common cancellation reason: Too Expensive (957 events).
-• Highest-risk segment: Consumer via Affiliate (368.8% cancelled share).
+• Highest-risk segment: Consumer via Partner (32.4% cancelled share).
 • Highest monthly churn: 2026-06 (3.19%).
 • Current recurring revenue: $371,044.95 MRR.
 • Main retention lesson: payment recovery, usage, product value, support, and cancellation intent require different interventions.</x:v>
@@ -1987,7 +1989,7 @@
     <x:mergeCell ref="A32:N38"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reef58d22edf04d05"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbee5a2179d9e4118"/>
 </x:worksheet>
 </file>
 
@@ -2138,7 +2140,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re463ebfb5ef24c49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94d5583e901540f7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3436,7 +3438,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6675a47d554e499e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35b4099d3cc54fc9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3680,7 +3682,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R129fbdd8d21c4051"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf973619566324407"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -3926,7 +3928,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8d884babbde47e9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3d73319092c4198"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -3992,25 +3994,25 @@
         <x:v>Consumer</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>Affiliate</x:v>
+        <x:v>Partner</x:v>
       </x:c>
       <x:c r="C2" t="n">
-        <x:v>990</x:v>
+        <x:v>704</x:v>
       </x:c>
       <x:c r="D2" t="n">
-        <x:v>3651</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="E2" s="10" t="n">
-        <x:v>3.687878787878788</x:v>
+        <x:v>0.323864</x:v>
       </x:c>
       <x:c r="F2" s="10" t="n">
-        <x:v>0.5261431329330394</x:v>
+        <x:v>0.534069</x:v>
       </x:c>
       <x:c r="G2" s="16" t="n">
-        <x:v>7.439841909249829</x:v>
+        <x:v>7.472393</x:v>
       </x:c>
       <x:c r="H2" s="12" t="n">
-        <x:v>362197.18</x:v>
+        <x:v>255203.39</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4018,25 +4020,25 @@
         <x:v>Consumer</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Paid Social</x:v>
+        <x:v>Affiliate</x:v>
       </x:c>
       <x:c r="C3" t="n">
-        <x:v>1961</x:v>
+        <x:v>990</x:v>
       </x:c>
       <x:c r="D3" t="n">
-        <x:v>6971</x:v>
+        <x:v>318</x:v>
       </x:c>
       <x:c r="E3" s="10" t="n">
-        <x:v>3.5548189699133097</x:v>
+        <x:v>0.321212</x:v>
       </x:c>
       <x:c r="F3" s="10" t="n">
-        <x:v>0.5229679136358388</x:v>
+        <x:v>0.526143</x:v>
       </x:c>
       <x:c r="G3" s="16" t="n">
-        <x:v>7.435977369818728</x:v>
+        <x:v>7.439842</x:v>
       </x:c>
       <x:c r="H3" s="12" t="n">
-        <x:v>712715.61</x:v>
+        <x:v>362197.18</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -4050,16 +4052,16 @@
         <x:v>1411</x:v>
       </x:c>
       <x:c r="D4" t="n">
-        <x:v>4932</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="E4" s="10" t="n">
-        <x:v>3.495393338058115</x:v>
+        <x:v>0.321049</x:v>
       </x:c>
       <x:c r="F4" s="10" t="n">
-        <x:v>0.5286165302267003</x:v>
+        <x:v>0.528617</x:v>
       </x:c>
       <x:c r="G4" s="16" t="n">
-        <x:v>7.450671704450042</x:v>
+        <x:v>7.450672</x:v>
       </x:c>
       <x:c r="H4" s="12" t="n">
         <x:v>523322.53</x:v>
@@ -4070,25 +4072,25 @@
         <x:v>Consumer</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Referral</x:v>
+        <x:v>Paid Social</x:v>
       </x:c>
       <x:c r="C5" t="n">
-        <x:v>1607</x:v>
+        <x:v>1961</x:v>
       </x:c>
       <x:c r="D5" t="n">
-        <x:v>5459</x:v>
+        <x:v>628</x:v>
       </x:c>
       <x:c r="E5" s="10" t="n">
-        <x:v>3.3970130678282513</x:v>
+        <x:v>0.320245</x:v>
       </x:c>
       <x:c r="F5" s="10" t="n">
-        <x:v>0.5297439288403615</x:v>
+        <x:v>0.522968</x:v>
       </x:c>
       <x:c r="G5" s="16" t="n">
-        <x:v>7.455948795180723</x:v>
+        <x:v>7.435977</x:v>
       </x:c>
       <x:c r="H5" s="12" t="n">
-        <x:v>591202.38</x:v>
+        <x:v>712715.61</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -4102,16 +4104,16 @@
         <x:v>2426</x:v>
       </x:c>
       <x:c r="D6" t="n">
-        <x:v>8219</x:v>
+        <x:v>773</x:v>
       </x:c>
       <x:c r="E6" s="10" t="n">
-        <x:v>3.387881286067601</x:v>
+        <x:v>0.318631</x:v>
       </x:c>
       <x:c r="F6" s="10" t="n">
-        <x:v>0.5228760931129991</x:v>
+        <x:v>0.522876</x:v>
       </x:c>
       <x:c r="G6" s="16" t="n">
-        <x:v>7.438614508449258</x:v>
+        <x:v>7.438615</x:v>
       </x:c>
       <x:c r="H6" s="12" t="n">
         <x:v>868169.55</x:v>
@@ -4119,54 +4121,54 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Premium Consumer</x:v>
+        <x:v>Consumer</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Partner</x:v>
+        <x:v>Referral</x:v>
       </x:c>
       <x:c r="C7" t="n">
-        <x:v>193</x:v>
+        <x:v>1607</x:v>
       </x:c>
       <x:c r="D7" t="n">
-        <x:v>646</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="E7" s="10" t="n">
-        <x:v>3.3471502590673574</x:v>
+        <x:v>0.316739</x:v>
       </x:c>
       <x:c r="F7" s="10" t="n">
-        <x:v>0.6953520912547528</x:v>
+        <x:v>0.529744</x:v>
       </x:c>
       <x:c r="G7" s="16" t="n">
-        <x:v>7.9638783269961975</x:v>
+        <x:v>7.455949</x:v>
       </x:c>
       <x:c r="H7" s="12" t="n">
-        <x:v>116811.07</x:v>
+        <x:v>591202.38</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>Small Business</x:v>
+        <x:v>Premium Consumer</x:v>
       </x:c>
       <x:c r="B8" t="str">
         <x:v>Direct</x:v>
       </x:c>
       <x:c r="C8" t="n">
-        <x:v>251</x:v>
+        <x:v>397</x:v>
       </x:c>
       <x:c r="D8" t="n">
-        <x:v>829</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="E8" s="10" t="n">
-        <x:v>3.302788844621514</x:v>
+        <x:v>0.284635</x:v>
       </x:c>
       <x:c r="F8" s="10" t="n">
-        <x:v>0.8083361966657248</x:v>
+        <x:v>0.700118</x:v>
       </x:c>
       <x:c r="G8" s="16" t="n">
-        <x:v>8.191296976547047</x:v>
+        <x:v>7.954857</x:v>
       </x:c>
       <x:c r="H8" s="12" t="n">
-        <x:v>280118.93</x:v>
+        <x:v>249918.48</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -4180,16 +4182,16 @@
         <x:v>415</x:v>
       </x:c>
       <x:c r="D9" t="n">
-        <x:v>1320</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="E9" s="10" t="n">
-        <x:v>3.180722891566265</x:v>
+        <x:v>0.281928</x:v>
       </x:c>
       <x:c r="F9" s="10" t="n">
-        <x:v>0.6954263549415515</x:v>
+        <x:v>0.695426</x:v>
       </x:c>
       <x:c r="G9" s="16" t="n">
-        <x:v>7.922954303931987</x:v>
+        <x:v>7.922954</x:v>
       </x:c>
       <x:c r="H9" s="12" t="n">
         <x:v>260806.61</x:v>
@@ -4206,16 +4208,16 @@
         <x:v>493</x:v>
       </x:c>
       <x:c r="D10" t="n">
-        <x:v>1560</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="E10" s="10" t="n">
-        <x:v>3.1643002028397564</x:v>
+        <x:v>0.275862</x:v>
       </x:c>
       <x:c r="F10" s="10" t="n">
-        <x:v>0.6978287215152411</x:v>
+        <x:v>0.697829</x:v>
       </x:c>
       <x:c r="G10" s="16" t="n">
-        <x:v>7.959899378514353</x:v>
+        <x:v>7.959899</x:v>
       </x:c>
       <x:c r="H10" s="12" t="n">
         <x:v>311202.12</x:v>
@@ -4223,28 +4225,28 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>Consumer</x:v>
+        <x:v>Premium Consumer</x:v>
       </x:c>
       <x:c r="B11" t="str">
         <x:v>Partner</x:v>
       </x:c>
       <x:c r="C11" t="n">
-        <x:v>704</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="D11" t="n">
-        <x:v>2210</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="E11" s="10" t="n">
-        <x:v>3.1392045454545454</x:v>
+        <x:v>0.274611</x:v>
       </x:c>
       <x:c r="F11" s="10" t="n">
-        <x:v>0.534068818741751</x:v>
+        <x:v>0.695352</x:v>
       </x:c>
       <x:c r="G11" s="16" t="n">
-        <x:v>7.472393312802463</x:v>
+        <x:v>7.963878</x:v>
       </x:c>
       <x:c r="H11" s="12" t="n">
-        <x:v>255203.39</x:v>
+        <x:v>116811.07</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -4258,16 +4260,16 @@
         <x:v>681</x:v>
       </x:c>
       <x:c r="D12" t="n">
-        <x:v>2131</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="E12" s="10" t="n">
-        <x:v>3.129221732745962</x:v>
+        <x:v>0.271659</x:v>
       </x:c>
       <x:c r="F12" s="10" t="n">
-        <x:v>0.6888621783876501</x:v>
+        <x:v>0.688862</x:v>
       </x:c>
       <x:c r="G12" s="16" t="n">
-        <x:v>7.916059176672384</x:v>
+        <x:v>7.916059</x:v>
       </x:c>
       <x:c r="H12" s="12" t="n">
         <x:v>413307.39</x:v>
@@ -4275,28 +4277,28 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>Premium Consumer</x:v>
+        <x:v>Small Business</x:v>
       </x:c>
       <x:c r="B13" t="str">
-        <x:v>Affiliate</x:v>
+        <x:v>Direct</x:v>
       </x:c>
       <x:c r="C13" t="n">
-        <x:v>272</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="D13" t="n">
-        <x:v>839</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="E13" s="10" t="n">
-        <x:v>3.0845588235294117</x:v>
+        <x:v>0.270916</x:v>
       </x:c>
       <x:c r="F13" s="10" t="n">
-        <x:v>0.701263959390863</x:v>
+        <x:v>0.808336</x:v>
       </x:c>
       <x:c r="G13" s="16" t="n">
-        <x:v>7.937750467539407</x:v>
+        <x:v>8.191297</x:v>
       </x:c>
       <x:c r="H13" s="12" t="n">
-        <x:v>174003.76</x:v>
+        <x:v>280118.93</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -4304,25 +4306,25 @@
         <x:v>Premium Consumer</x:v>
       </x:c>
       <x:c r="B14" t="str">
-        <x:v>Direct</x:v>
+        <x:v>Affiliate</x:v>
       </x:c>
       <x:c r="C14" t="n">
-        <x:v>397</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="D14" t="n">
-        <x:v>1179</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="E14" s="10" t="n">
-        <x:v>2.9697732997481108</x:v>
+        <x:v>0.264706</x:v>
       </x:c>
       <x:c r="F14" s="10" t="n">
-        <x:v>0.7001181498612397</x:v>
+        <x:v>0.701264</x:v>
       </x:c>
       <x:c r="G14" s="16" t="n">
-        <x:v>7.954856614246069</x:v>
+        <x:v>7.93775</x:v>
       </x:c>
       <x:c r="H14" s="12" t="n">
-        <x:v>249918.48</x:v>
+        <x:v>174003.76</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -4336,16 +4338,16 @@
         <x:v>326</x:v>
       </x:c>
       <x:c r="D15" t="n">
-        <x:v>948</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="E15" s="10" t="n">
-        <x:v>2.9079754601226995</x:v>
+        <x:v>0.242331</x:v>
       </x:c>
       <x:c r="F15" s="10" t="n">
-        <x:v>0.7911583839229642</x:v>
+        <x:v>0.791158</x:v>
       </x:c>
       <x:c r="G15" s="16" t="n">
-        <x:v>8.159933012350848</x:v>
+        <x:v>8.159933</x:v>
       </x:c>
       <x:c r="H15" s="12" t="n">
         <x:v>358713.13</x:v>
@@ -4356,25 +4358,25 @@
         <x:v>Small Business</x:v>
       </x:c>
       <x:c r="B16" t="str">
-        <x:v>Referral</x:v>
+        <x:v>Organic Search</x:v>
       </x:c>
       <x:c r="C16" t="n">
-        <x:v>275</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="D16" t="n">
-        <x:v>718</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="E16" s="10" t="n">
-        <x:v>2.610909090909091</x:v>
+        <x:v>0.220264</x:v>
       </x:c>
       <x:c r="F16" s="10" t="n">
-        <x:v>0.79608023744744</x:v>
+        <x:v>0.798521</x:v>
       </x:c>
       <x:c r="G16" s="16" t="n">
-        <x:v>8.215186742517933</x:v>
+        <x:v>8.154799</x:v>
       </x:c>
       <x:c r="H16" s="12" t="n">
-        <x:v>320453.21</x:v>
+        <x:v>501157.78</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -4382,25 +4384,25 @@
         <x:v>Small Business</x:v>
       </x:c>
       <x:c r="B17" t="str">
-        <x:v>Organic Search</x:v>
+        <x:v>Referral</x:v>
       </x:c>
       <x:c r="C17" t="n">
-        <x:v>454</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="D17" t="n">
-        <x:v>1102</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="E17" s="10" t="n">
-        <x:v>2.4273127753303965</x:v>
+        <x:v>0.210909</x:v>
       </x:c>
       <x:c r="F17" s="10" t="n">
-        <x:v>0.7985208751568381</x:v>
+        <x:v>0.79608</x:v>
       </x:c>
       <x:c r="G17" s="16" t="n">
-        <x:v>8.154799247176914</x:v>
+        <x:v>8.215187</x:v>
       </x:c>
       <x:c r="H17" s="12" t="n">
-        <x:v>501157.78</x:v>
+        <x:v>320453.21</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -4408,25 +4410,25 @@
         <x:v>Small Business</x:v>
       </x:c>
       <x:c r="B18" t="str">
-        <x:v>Affiliate</x:v>
+        <x:v>Partner</x:v>
       </x:c>
       <x:c r="C18" t="n">
-        <x:v>171</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="D18" t="n">
-        <x:v>362</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E18" s="10" t="n">
-        <x:v>2.1169590643274856</x:v>
+        <x:v>0.20155</x:v>
       </x:c>
       <x:c r="F18" s="10" t="n">
-        <x:v>0.8063114425827544</x:v>
+        <x:v>0.807842</x:v>
       </x:c>
       <x:c r="G18" s="16" t="n">
-        <x:v>8.209644462607274</x:v>
+        <x:v>8.189158</x:v>
       </x:c>
       <x:c r="H18" s="12" t="n">
-        <x:v>202100.75</x:v>
+        <x:v>139647.02</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -4434,25 +4436,25 @@
         <x:v>Small Business</x:v>
       </x:c>
       <x:c r="B19" t="str">
-        <x:v>Partner</x:v>
+        <x:v>Affiliate</x:v>
       </x:c>
       <x:c r="C19" t="n">
-        <x:v>129</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="D19" t="n">
-        <x:v>263</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="E19" s="10" t="n">
-        <x:v>2.0387596899224807</x:v>
+        <x:v>0.169591</x:v>
       </x:c>
       <x:c r="F19" s="10" t="n">
-        <x:v>0.8078418685121107</x:v>
+        <x:v>0.806311</x:v>
       </x:c>
       <x:c r="G19" s="16" t="n">
-        <x:v>8.189158016147635</x:v>
+        <x:v>8.209644</x:v>
       </x:c>
       <x:c r="H19" s="12" t="n">
-        <x:v>139647.02</x:v>
+        <x:v>202100.75</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4470,7 +4472,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2014532d7ed949c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R834415c27b75439f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10523,7 +10525,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa014a89e7954d64"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c684943e9b64d11"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10650,7 +10652,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e9b4783dab04740"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc14c5ba5301449db"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>